<commit_message>
Upload Form Material Request Metalurgy dan Gold Room 31 Oktober 2026.xlsx via Zeta Client · 59 sel berubah · F_Material Request
</commit_message>
<xml_diff>
--- a/Form_PO_Barang/Form Material Request Metalurgy dan Gold Room 31 Oktober 2026.xlsx
+++ b/Form_PO_Barang/Form Material Request Metalurgy dan Gold Room 31 Oktober 2026.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dyanr\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramda\Documents\Zeta_Edit\7b5b69b8bcd7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40B61931-DBB7-43AE-9193-B538F2BE6BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D802EA65-8BC3-44FC-B71B-8373BE39B3B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="F_Material Request" sheetId="3" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'F_Material Request'!$A$1:$I$31</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'F_Material Request'!$A$1:$I$34</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="67">
   <si>
     <t xml:space="preserve">NO </t>
   </si>
@@ -371,9 +371,6 @@
     </r>
   </si>
   <si>
-    <t>Tanggal Dibutuhkan : 26/ 10  / 2026</t>
-  </si>
-  <si>
     <t>Pcs</t>
   </si>
   <si>
@@ -383,9 +380,6 @@
     <t>Unit</t>
   </si>
   <si>
-    <t>Kristian Djalimun</t>
-  </si>
-  <si>
     <t>Tanggal : 31/10/2026</t>
   </si>
   <si>
@@ -459,6 +453,42 @@
   </si>
   <si>
     <t>https://www.tokopedia.com/pramuka-jakartapt/buchner-funnel-100-mm-corong-porselen</t>
+  </si>
+  <si>
+    <t>Timbangan duduk digital</t>
+  </si>
+  <si>
+    <t>max 35 Kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pipa PVC </t>
+  </si>
+  <si>
+    <t>4 meter, 1 inch</t>
+  </si>
+  <si>
+    <t>pcs</t>
+  </si>
+  <si>
+    <t>untuk jalur flushing line carbon  outlet electrowinning</t>
+  </si>
+  <si>
+    <t>Elbow PVC</t>
+  </si>
+  <si>
+    <t>1 inch</t>
+  </si>
+  <si>
+    <t>Water mur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">untuk menimbang sample dari pabrik dan Test work </t>
+  </si>
+  <si>
+    <t>Tanggal Dibutuhkan : 02 / 11  / 2026</t>
+  </si>
+  <si>
+    <t>Nama : Kristian Djalimun</t>
   </si>
 </sst>
 </file>
@@ -734,7 +764,7 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -802,22 +832,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -833,27 +863,57 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma [0]" xfId="1" builtinId="6"/>
@@ -929,14 +989,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>21</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>155678</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>272921</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>160287</xdr:rowOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>160286</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1003,9 +1063,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1043,9 +1103,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1078,26 +1138,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1130,26 +1173,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1326,25 +1352,25 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M31"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:M34"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.54296875" style="3" customWidth="1"/>
-    <col min="2" max="2" width="6.81640625" customWidth="1"/>
-    <col min="3" max="3" width="11.36328125" customWidth="1"/>
-    <col min="4" max="4" width="13.81640625" customWidth="1"/>
-    <col min="5" max="5" width="26.453125" customWidth="1"/>
-    <col min="6" max="6" width="6.08984375" customWidth="1"/>
-    <col min="7" max="7" width="31.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="29.1796875" customWidth="1"/>
-    <col min="10" max="10" width="16.08984375" customWidth="1"/>
-    <col min="11" max="11" width="22.6328125" customWidth="1"/>
+    <col min="1" max="1" width="4.5546875" style="3" customWidth="1"/>
+    <col min="2" max="2" width="6.77734375" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" customWidth="1"/>
+    <col min="5" max="5" width="26.44140625" customWidth="1"/>
+    <col min="6" max="6" width="6.109375" customWidth="1"/>
+    <col min="7" max="7" width="31.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="46.6640625" customWidth="1"/>
+    <col min="10" max="10" width="16.109375" customWidth="1"/>
+    <col min="11" max="11" width="22.6640625" customWidth="1"/>
     <col min="12" max="12" width="22" customWidth="1"/>
-    <col min="13" max="13" width="57.90625" customWidth="1"/>
+    <col min="13" max="13" width="57.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="19" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:13" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D1" s="33" t="s">
         <v>2</v>
       </c>
@@ -1358,7 +1384,7 @@
       <c r="L1" s="4"/>
       <c r="M1" s="4"/>
     </row>
-    <row r="2" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5"/>
       <c r="B2" s="5"/>
       <c r="C2" s="6"/>
@@ -1377,7 +1403,7 @@
       <c r="L2" s="5"/>
       <c r="M2" s="5"/>
     </row>
-    <row r="3" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3"/>
       <c r="D3" s="36" t="s">
         <v>25</v>
@@ -1388,10 +1414,10 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4"/>
       <c r="D4" s="36" t="s">
-        <v>27</v>
+        <v>65</v>
       </c>
       <c r="E4" s="36"/>
       <c r="F4" s="36"/>
@@ -1402,7 +1428,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="D5" s="36" t="s">
         <v>26</v>
@@ -1413,7 +1439,7 @@
       <c r="H5" s="36"/>
       <c r="I5" s="36"/>
     </row>
-    <row r="6" spans="1:13" ht="16.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="D6" s="25"/>
       <c r="E6" s="26"/>
@@ -1424,7 +1450,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:13" s="9" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" s="9" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
         <v>0</v>
       </c>
@@ -1453,335 +1479,418 @@
       <c r="L7" s="7"/>
       <c r="M7" s="8"/>
     </row>
-    <row r="8" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="14">
         <v>1</v>
       </c>
-      <c r="B8" s="38" t="s">
+      <c r="B8" s="39" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="40"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="54" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" s="27">
+        <v>100</v>
+      </c>
+      <c r="G8" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="39"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="29" t="s">
+      <c r="H8" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="I8" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="1">
-        <v>100</v>
-      </c>
-      <c r="G8" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I8" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="J8" s="30" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="32.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J8" s="28" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="14">
         <v>2</v>
       </c>
-      <c r="B9" s="38" t="s">
-        <v>55</v>
-      </c>
-      <c r="C9" s="39"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F9" s="1">
+      <c r="B9" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="40"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="F9" s="27">
         <v>3</v>
       </c>
-      <c r="G9" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="I9" s="31" t="s">
-        <v>41</v>
-      </c>
-      <c r="J9" s="30" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G9" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="27" t="s">
+        <v>38</v>
+      </c>
+      <c r="I9" s="51" t="s">
+        <v>39</v>
+      </c>
+      <c r="J9" s="28" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14">
         <v>3</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="42" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="43"/>
+      <c r="D10" s="44"/>
+      <c r="E10" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="F10" s="27">
+        <v>3</v>
+      </c>
+      <c r="G10" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="38" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="42"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="1" t="s">
+      <c r="I10" s="51" t="s">
         <v>39</v>
       </c>
-      <c r="F10" s="1">
-        <v>3</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H10" s="31" t="s">
-        <v>40</v>
-      </c>
-      <c r="I10" s="31" t="s">
-        <v>41</v>
-      </c>
-      <c r="J10" s="30" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="J10" s="28" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="14">
         <v>4</v>
       </c>
-      <c r="B11" s="41" t="s">
+      <c r="B11" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="43"/>
+      <c r="D11" s="44"/>
+      <c r="E11" s="54" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" s="27">
+        <v>1</v>
+      </c>
+      <c r="G11" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="42"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="31" t="s">
+      <c r="H11" s="27" t="s">
+        <v>38</v>
+      </c>
+      <c r="I11" s="51" t="s">
+        <v>39</v>
+      </c>
+      <c r="J11" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="F11" s="1">
-        <v>1</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="I11" s="31" t="s">
-        <v>41</v>
-      </c>
-      <c r="J11" s="30" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="14">
         <v>5</v>
       </c>
-      <c r="B12" s="44" t="s">
-        <v>48</v>
-      </c>
-      <c r="C12" s="45"/>
-      <c r="D12" s="46"/>
-      <c r="E12" s="31" t="s">
-        <v>53</v>
-      </c>
-      <c r="F12" s="1">
+      <c r="B12" s="45" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="46"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="54" t="s">
+        <v>51</v>
+      </c>
+      <c r="F12" s="27">
         <v>5</v>
       </c>
-      <c r="G12" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H12" s="1" t="s">
+      <c r="G12" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="I12" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="H12" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="I12" s="53" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="14">
         <v>6</v>
       </c>
-      <c r="B13" s="44" t="s">
+      <c r="B13" s="45" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" s="46"/>
+      <c r="D13" s="47"/>
+      <c r="E13" s="54" t="s">
+        <v>49</v>
+      </c>
+      <c r="F13" s="27">
+        <v>1</v>
+      </c>
+      <c r="G13" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="H13" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="I13" s="51" t="s">
         <v>50</v>
       </c>
-      <c r="C13" s="45"/>
-      <c r="D13" s="46"/>
-      <c r="E13" s="31" t="s">
-        <v>51</v>
-      </c>
-      <c r="F13" s="1">
-        <v>1</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I13" s="31" t="s">
-        <v>52</v>
-      </c>
-      <c r="J13" s="30" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J13" s="28" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="14">
         <v>7</v>
       </c>
-      <c r="B14" s="15"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-    </row>
-    <row r="15" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="42" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" s="43"/>
+      <c r="D14" s="44"/>
+      <c r="E14" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="F14" s="27">
+        <v>2</v>
+      </c>
+      <c r="G14" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="H14" s="27" t="s">
+        <v>38</v>
+      </c>
+      <c r="I14" s="53" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="14">
         <v>8</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-    </row>
-    <row r="16" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="48" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" s="49"/>
+      <c r="D15" s="50"/>
+      <c r="E15" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="F15" s="27">
+        <v>1</v>
+      </c>
+      <c r="G15" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="H15" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="I15" s="51" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="14">
         <v>9</v>
       </c>
-      <c r="B16" s="15"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-    </row>
-    <row r="17" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="30" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="31"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="F16" s="27">
+        <v>4</v>
+      </c>
+      <c r="G16" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="H16" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="I16" s="51" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="14">
         <v>10</v>
       </c>
-      <c r="B17" s="15"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-    </row>
-    <row r="19" spans="1:9" ht="16.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="34" t="s">
+      <c r="B17" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" s="31"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="F17" s="27">
+        <v>4</v>
+      </c>
+      <c r="G17" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="H17" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="I17" s="51" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="14">
+        <v>11</v>
+      </c>
+      <c r="B18" s="15"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+    </row>
+    <row r="19" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="14">
+        <v>12</v>
+      </c>
+      <c r="B19" s="15"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+    </row>
+    <row r="20" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="14">
         <v>13</v>
       </c>
-      <c r="B19" s="34"/>
-      <c r="C19" s="24" t="s">
+      <c r="B20" s="15"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+    </row>
+    <row r="22" spans="1:9" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="34" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22" s="34"/>
+      <c r="C22" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="24"/>
-    </row>
-    <row r="20" spans="1:9" ht="16.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="24"/>
-      <c r="B20" s="24"/>
-      <c r="C20" s="24" t="s">
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="24"/>
+    </row>
+    <row r="23" spans="1:9" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="24"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
-      <c r="I20" s="24"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A22" s="10" t="s">
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="24"/>
+      <c r="I23" s="24"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D25" t="s">
         <v>15</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G25" t="s">
         <v>12</v>
       </c>
-      <c r="I22" t="s">
+      <c r="I25" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A27" s="11" t="s">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="12"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="11" t="s">
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="E27" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="F27" s="12"/>
-      <c r="G27" s="11" t="s">
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="H30" s="12"/>
+      <c r="I30" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H27" s="12"/>
-      <c r="I27" s="11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A28" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B28" s="12"/>
-      <c r="C28" s="12"/>
-      <c r="D28" s="11" t="s">
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31" s="12"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E28" s="32">
-        <v>46326</v>
-      </c>
-      <c r="F28" s="12"/>
-      <c r="G28" s="11" t="s">
+      <c r="E31" s="29"/>
+      <c r="F31" s="12"/>
+      <c r="G31" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="H31" s="12"/>
+      <c r="I31" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="H28" s="12"/>
-      <c r="I28" s="11" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A30" s="18" t="s">
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="B30" s="19"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="19"/>
-      <c r="H30" s="19"/>
-      <c r="I30" s="20"/>
-    </row>
-    <row r="31" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="21"/>
-      <c r="B31" s="22"/>
-      <c r="C31" s="22"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
-      <c r="G31" s="22"/>
-      <c r="H31" s="22"/>
-      <c r="I31" s="23"/>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="19"/>
+      <c r="G33" s="19"/>
+      <c r="H33" s="19"/>
+      <c r="I33" s="20"/>
+    </row>
+    <row r="34" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="21"/>
+      <c r="B34" s="22"/>
+      <c r="C34" s="22"/>
+      <c r="D34" s="22"/>
+      <c r="E34" s="22"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="22"/>
+      <c r="H34" s="22"/>
+      <c r="I34" s="23"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
     <mergeCell ref="D1:I1"/>
-    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A22:B22"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="D5:I5"/>
     <mergeCell ref="D4:F4"/>
@@ -1794,6 +1903,7 @@
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B14:D14"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="J11" r:id="rId1" xr:uid="{6F6C0238-017B-4653-ACBD-AD7A64A7DBFA}"/>

</xml_diff>